<commit_message>
Update - but the PCB no work :(
</commit_message>
<xml_diff>
--- a/Documentation/WYVERN_E4_BOM.xlsx
+++ b/Documentation/WYVERN_E4_BOM.xlsx
@@ -588,7 +588,7 @@
     <t xml:space="preserve">RP2350B flight computer board</t>
   </si>
   <si>
-    <t xml:space="preserve">DFM-reviewed Gerber submission (soldermask/silkscreen/SMT placement flags addressed). $200 total for 3 fabricated boards (updated 2026-08-10, was $195); one of the three is earmarked for the ground servo TVC test stand rather than flight/spare use.</t>
+    <t xml:space="preserve">DFM-reviewed Gerber submission (soldermask/silkscreen/SMT placement flags addressed). $207.01 total for 3 fabricated boards (updated 2026-08-11, was $200); one of the three is earmarked for the ground servo TVC test stand rather than flight/spare use.</t>
   </si>
   <si>
     <t xml:space="preserve">eMagTech F-F servo extension cable 10cm (10-pk)</t>
@@ -3592,7 +3592,7 @@
       <c r="G96" s="18"/>
       <c r="H96" s="19" t="n">
         <f aca="false">H11+H21+H29+H37+H47+H56+H84+H94+H111+H124</f>
-        <v>1206.58</v>
+        <v>1213.59</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3616,7 +3616,7 @@
       <c r="G98" s="18"/>
       <c r="H98" s="23" t="n">
         <f aca="false">H96+H97</f>
-        <v>1166.98</v>
+        <v>1173.99</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3671,11 +3671,11 @@
         <v>3</v>
       </c>
       <c r="G102" s="1" t="n">
-        <v>66.6666666666667</v>
+        <v>69.0033333333333</v>
       </c>
       <c r="H102" s="1" t="n">
         <f aca="false">F102*G102</f>
-        <v>200</v>
+        <v>207.01</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3900,7 +3900,7 @@
       </c>
       <c r="H111" s="1" t="n">
         <f aca="false">SUM(H102:H110)</f>
-        <v>293.43</v>
+        <v>300.44</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5046,7 +5046,7 @@
       </c>
       <c r="B11" s="1" t="n">
         <f aca="false">BOM!H111</f>
-        <v>293.43</v>
+        <v>300.44</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="B13" s="30" t="n">
         <f aca="false">BOM!H96</f>
-        <v>1206.58</v>
+        <v>1213.59</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5082,7 +5082,7 @@
       </c>
       <c r="B15" s="32" t="n">
         <f aca="false">BOM!H98</f>
-        <v>1166.98</v>
+        <v>1173.99</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -5101,7 +5101,7 @@
       </c>
       <c r="B18" s="28" t="n">
         <f aca="false">B15+B17</f>
-        <v>1646.25</v>
+        <v>1653.26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>